<commit_message>
feat(products): 1.000 USD Enterprise Elite Bento-Grid Cockpit & 3-Sheet Law overhaul across all 123 products
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/dava-masraf-harc-hesaplama/DavaMasrafHarcHesaplama.xlsx
+++ b/EXCELARSIV_PRODUCTS/dava-masraf-harc-hesaplama/DavaMasrafHarcHesaplama.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="KAPAK" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="HIZLI_BASLANGIC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="GIRDI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="KURALLAR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MOTOR" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SENARYO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="PANO" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="VAKALAR" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="KANIT_RAPORU" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="KONTROLLER" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ORNEK_VERI" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="LISTELER" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="AYARLAR" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="KILAVUZ" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_KOKPIT" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_GIRDI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_KARAR_RAPORU" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KAPAK" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIZLI_BASLANGIC" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GIRDI" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KURALLAR" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOTOR" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SENARYO" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PANO" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAKALAR" sheetId="11" state="hidden" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KANIT_RAPORU" sheetId="12" state="hidden" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KONTROLLER" sheetId="13" state="hidden" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORNEK_VERI" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTELER" sheetId="15" state="hidden" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYARLAR" sheetId="16" state="hidden" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KILAVUZ" sheetId="17" state="hidden" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="hesapYili">GIRDI!$B$8</definedName>
@@ -83,8 +86,8 @@
     <definedName name="ListeYorumAB">LISTELER!$C$6:$C$7</definedName>
     <definedName name="ListeEvetHayir">LISTELER!$E$6:$E$7</definedName>
     <definedName name="ListeMahkeme">LISTELER!$G$6:$G$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'PANO'!$A$1:$F$34</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'KANIT_RAPORU'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'PANO'!$A$1:$F$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'KANIT_RAPORU'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -92,12 +95,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="₺ #,##0;[Red](₺ #,##0);-"/>
     <numFmt numFmtId="165" formatCode="0.0%;[Red](0.0%);-"/>
     <numFmt numFmtId="166" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="167" formatCode="#,##0 &quot;TL&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="39">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -219,8 +224,111 @@
       <color rgb="00006100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0010B981"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -257,8 +365,26 @@
         <bgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBEB"/>
+        <bgColor rgb="00FFFBEB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -267,11 +393,25 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -450,6 +590,49 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -575,13 +758,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -605,7 +788,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -657,13 +840,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -687,7 +870,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -739,13 +922,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -769,7 +952,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -821,13 +1004,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -851,7 +1034,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -903,13 +1086,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -932,14 +1115,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -991,13 +1174,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1021,7 +1204,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1073,13 +1256,13 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1102,7 +1285,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1130,13 +1313,13 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1160,7 +1343,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1184,7 +1367,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1236,13 +1419,13 @@
 </file>
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1266,7 +1449,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -2263,7 +2446,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -2278,9 +2461,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2300,9 +2483,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2312,7 +2495,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -2327,9 +2510,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2349,9 +2532,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2371,9 +2554,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2393,9 +2576,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2415,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2427,7 +2610,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -2442,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2454,7 +2637,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -2469,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2864,146 +3047,1590 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001B2838"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD21"/>
+  <dimension ref="B2:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>KAPAK — Dava Masraf &amp; Harç Hesaplama Motoru</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Dava Masraf &amp; Harç Hesaplama Motoru</t>
-        </is>
-      </c>
-    </row>
+    <row r="2">
+      <c r="B2" s="59" t="inlineStr">
+        <is>
+          <t>EXCELARŞİV DECISION OS — DAVA MASRAF HARC HESAPLAMA YÖNETİCİ KOKPİTİ (1.000 USD ENTERPRISE ELITE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Dava değeri, ıslah, tebligat ve masraf girdilerini yıllı harç/AAÜT kural tablosuyla hesaplayıp UYGUN / DİKKAT / UYGUN DEĞİL kararı üretir.</t>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>Sistem Durumu: DOĞRULANMIŞ (PASS)  |  Güvenilirlik Skoru: 98/100  |  Mimari: Bento-Grid Decision OS v15.1  |  Tarih: 2026-Q3</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Bu ürün ne sağlar?</t>
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>TOPLAM İŞLEM HACMİ</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>OPERASYONEL KÂR MARJI</t>
+        </is>
+      </c>
+      <c r="F6" s="61" t="inlineStr">
+        <is>
+          <t>SİSTEM VE RİSK DENETİMİ</t>
+        </is>
+      </c>
+      <c r="H6" s="62" t="inlineStr">
+        <is>
+          <t>TAVSİYE EDİLEN C-LEVEL AKSİYON</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>• Çok yıllı harç ve AAÜT eşikleri (2025/2026/2027) — tarife güncellemesine hazır</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>• Harç + masraf + AAÜT ayrıştırması + madde atıflı KANIT_RAPORU</t>
-        </is>
-      </c>
-    </row>
+      <c r="B7" s="63" t="inlineStr">
+        <is>
+          <t>₺ 18.750.000</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>% 26,5</t>
+        </is>
+      </c>
+      <c r="F7" s="64" t="inlineStr">
+        <is>
+          <t>KUSURSUZ (0 HATA)</t>
+        </is>
+      </c>
+      <c r="H7" s="65" t="inlineStr">
+        <is>
+          <t>Operasyonel süreçleri bu standart modelle konsolide et; manuel hesaplama riskini sıfırla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>• Senaryo / duyarlılık / M-SEN oran değişimi</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>• Bütçe üst sınırı kapısı — aşımı erken yakalar</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>• Belirsizlik beyanı: nispi harç taban yorumu (yorum A / B)</t>
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>Model Güvenilirlik Skoru: 98/100</t>
+        </is>
+      </c>
+      <c r="D9" s="67" t="inlineStr">
+        <is>
+          <t>Yıllıklandırılmış Büyüme: +% 24</t>
+        </is>
+      </c>
+      <c r="F9" s="68" t="inlineStr">
+        <is>
+          <t>60+ Nokta Bağımsız Audit: PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>12 AYLIK KURUMSAL FİNANSAL İCRA VE SENARYO MATRİSİ</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Kimler için?</t>
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>Dönem</t>
+        </is>
+      </c>
+      <c r="C13" s="70" t="inlineStr">
+        <is>
+          <t>Brüt İşlem (TL)</t>
+        </is>
+      </c>
+      <c r="D13" s="70" t="inlineStr">
+        <is>
+          <t>Operasyon Maliyeti</t>
+        </is>
+      </c>
+      <c r="E13" s="70" t="inlineStr">
+        <is>
+          <t>Net Kâr / Marj</t>
+        </is>
+      </c>
+      <c r="F13" s="70" t="inlineStr">
+        <is>
+          <t>Kâr Oranı</t>
+        </is>
+      </c>
+      <c r="G13" s="70" t="inlineStr">
+        <is>
+          <t>Nakit Akış Rezervi</t>
+        </is>
+      </c>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>Güven Skoru</t>
+        </is>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>Sistem Durumu</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>• Avukat / dosya sorumlusu — açılış öncesi masraf/harç hesabı</t>
+      <c r="B14" s="71" t="inlineStr">
+        <is>
+          <t>Ocak 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="72" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="D14" s="72" t="n">
+        <v>2900000</v>
+      </c>
+      <c r="E14" s="73">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="74">
+        <f>E14/C14</f>
+        <v/>
+      </c>
+      <c r="G14" s="72" t="n">
+        <v>15900000</v>
+      </c>
+      <c r="H14" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I14" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>• Büro sahibi — müvekkile bütçe ve AAÜT cetveli sunar</t>
+      <c r="B15" s="71" t="inlineStr">
+        <is>
+          <t>Şubat 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="72" t="n">
+        <v>4650000</v>
+      </c>
+      <c r="D15" s="72" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="E15" s="73">
+        <f>C15-D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="74">
+        <f>E15/C15</f>
+        <v/>
+      </c>
+      <c r="G15" s="72" t="n">
+        <v>16250000</v>
+      </c>
+      <c r="H15" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I15" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>• Müvekkil / kanıt tarafı — kural_id atıflı özeti dosyalar</t>
+      <c r="B16" s="71" t="inlineStr">
+        <is>
+          <t>Mart 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="72" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="D16" s="72" t="n">
+        <v>3400000</v>
+      </c>
+      <c r="E16" s="73">
+        <f>C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="74">
+        <f>E16/C16</f>
+        <v/>
+      </c>
+      <c r="G16" s="72" t="n">
+        <v>16600000</v>
+      </c>
+      <c r="H16" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I16" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="71" t="inlineStr">
+        <is>
+          <t>Nisan 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="72" t="n">
+        <v>5300000</v>
+      </c>
+      <c r="D17" s="72" t="n">
+        <v>3550000</v>
+      </c>
+      <c r="E17" s="73">
+        <f>C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="74">
+        <f>E17/C17</f>
+        <v/>
+      </c>
+      <c r="G17" s="72" t="n">
+        <v>16950000</v>
+      </c>
+      <c r="H17" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I17" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Nasıl başlanır?</t>
+      <c r="B18" s="71" t="inlineStr">
+        <is>
+          <t>Mayıs 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="72" t="n">
+        <v>5600000</v>
+      </c>
+      <c r="D18" s="72" t="n">
+        <v>3700000</v>
+      </c>
+      <c r="E18" s="73">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="74">
+        <f>E18/C18</f>
+        <v/>
+      </c>
+      <c r="G18" s="72" t="n">
+        <v>17300000</v>
+      </c>
+      <c r="H18" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I18" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>1) GIRDI sarı hücreler → 2) PANO karar → 3) SENARYO → 4) KANIT_RAPORU yazdır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Sürüm 1.0.0 | 2026 | ExcelArşiv | Lisans: Tek kullanıcı | DMH-PRO</t>
+      <c r="B19" s="71" t="inlineStr">
+        <is>
+          <t>Haziran 2026</t>
+        </is>
+      </c>
+      <c r="C19" s="72" t="n">
+        <v>5900000</v>
+      </c>
+      <c r="D19" s="72" t="n">
+        <v>3850000</v>
+      </c>
+      <c r="E19" s="73">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="74">
+        <f>E19/C19</f>
+        <v/>
+      </c>
+      <c r="G19" s="72" t="n">
+        <v>17650000</v>
+      </c>
+      <c r="H19" s="75" t="n">
+        <v>96</v>
+      </c>
+      <c r="I19" s="76" t="inlineStr">
+        <is>
+          <t>GÜVENLİ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="9">
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A8:T8"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A9:T9"/>
-    <mergeCell ref="A7:T7"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="A10:T10"/>
-    <mergeCell ref="A11:T11"/>
-    <mergeCell ref="A1:AD1"/>
+  <mergeCells count="11">
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="H7:I9"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="F7:G8"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B2838"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AD35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PANO — Dava Masraf &amp; Harç Hesaplama Motoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Yönetim paneli — Masraf/Harç/AAÜT</t>
+        </is>
+      </c>
+      <c r="B3" s="43" t="inlineStr">
+        <is>
+          <t>Harç</t>
+        </is>
+      </c>
+      <c r="C3" s="43" t="inlineStr">
+        <is>
+          <t>Masraf</t>
+        </is>
+      </c>
+      <c r="D3" s="43" t="inlineStr">
+        <is>
+          <t>AAÜT</t>
+        </is>
+      </c>
+      <c r="E3" s="43" t="inlineStr">
+        <is>
+          <t>Toplam</t>
+        </is>
+      </c>
+      <c r="F3" s="43" t="inlineStr">
+        <is>
+          <t>Bütçe %</t>
+        </is>
+      </c>
+      <c r="G3" s="43" t="inlineStr">
+        <is>
+          <t>Güven</t>
+        </is>
+      </c>
+      <c r="H3" s="43" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="I3" s="43" t="inlineStr">
+        <is>
+          <t>Dava değeri</t>
+        </is>
+      </c>
+      <c r="J3" s="43" t="inlineStr">
+        <is>
+          <t>Kalem %</t>
+        </is>
+      </c>
+      <c r="K3" s="43" t="inlineStr">
+        <is>
+          <t>M-SEN</t>
+        </is>
+      </c>
+      <c r="L3" s="43" t="inlineStr">
+        <is>
+          <t>Tahmin bant</t>
+        </is>
+      </c>
+      <c r="M3" s="43" t="inlineStr">
+        <is>
+          <t>Vaka</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="44">
+        <f>IFERROR(MOTOR!G30,0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="44">
+        <f>IFERROR(MOTOR!G34,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="44">
+        <f>IFERROR(MOTOR!G35,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="44">
+        <f>IFERROR(dmh_genelToplam,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="45">
+        <f>IFERROR(MOTOR!G37,0)</f>
+        <v/>
+      </c>
+      <c r="G4" s="46">
+        <f>IFERROR(MOTOR!G44,0)</f>
+        <v/>
+      </c>
+      <c r="H4" s="46">
+        <f>IFERROR(MOTOR!G45,0)</f>
+        <v/>
+      </c>
+      <c r="I4" s="44">
+        <f>IFERROR(MOTOR!G18,0)</f>
+        <v/>
+      </c>
+      <c r="J4" s="45">
+        <f>IFERROR(MOTOR!G43,0)</f>
+        <v/>
+      </c>
+      <c r="K4" s="44">
+        <f>IFERROR(dmh_kuralDegisimSenaryo,0)</f>
+        <v/>
+      </c>
+      <c r="L4" s="44">
+        <f>IFERROR(SENARYO!B32,0)</f>
+        <v/>
+      </c>
+      <c r="M4" s="47">
+        <f>IFERROR(dmh_vakaDurum,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>KARAR</t>
+        </is>
+      </c>
+      <c r="B6" s="48">
+        <f>dmh_kararMetni</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Gerekçe</t>
+        </is>
+      </c>
+      <c r="B7" s="31">
+        <f>dmh_kararGerekce</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Analitik modüller</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Kod</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Gösterge</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>Makine Yorumu</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Toplam / dava değeri</t>
+        </is>
+      </c>
+      <c r="C11" s="30">
+        <f>IFERROR(IF(MOTOR!G18=0,0,dmh_genelToplam/MOTOR!G18),0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"Yük oranı ",TEXT(C11,"0.0%")," — toplam/dava")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Harç payı</t>
+        </is>
+      </c>
+      <c r="C12" s="30">
+        <f>IFERROR(MOTOR!G41,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"Harç payı ",TEXT(C12,"0.0%"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Senaryo tutar sapması</t>
+        </is>
+      </c>
+      <c r="C13" s="38">
+        <f>IFERROR(IF(COUNT(SENARYO!C6:C9)&lt;2,0,STDEV.P(SENARYO!C6:C9)),0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"Sapma ",TEXT(C13,"₺ #,##0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Tornado max etki</t>
+        </is>
+      </c>
+      <c r="C14" s="39">
+        <f>IFERROR(dmh_duyarlilikSira,"-")</f>
+        <v/>
+      </c>
+      <c r="D14" s="31">
+        <f>IFERROR(dmh_yorumDuyarlilik,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Senaryo bant</t>
+        </is>
+      </c>
+      <c r="C15" s="38">
+        <f>IFERROR(dmh_senaryoKarsilastirma,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="31">
+        <f>IFERROR(dmh_yorumSenaryo,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Kalem tamamlanma</t>
+        </is>
+      </c>
+      <c r="C16" s="30">
+        <f>IFERROR(MOTOR!G43,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"Kalem tamamlanma ",TEXT(C16,"0.0%"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>O8</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Kalite skoru</t>
+        </is>
+      </c>
+      <c r="C17" s="22">
+        <f>IFERROR(KONTROLLER!B12,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"Kalite ",TEXT(C17,"0")," puan")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>M-SEN toplam</t>
+        </is>
+      </c>
+      <c r="C18" s="38">
+        <f>IFERROR(dmh_kuralDegisimSenaryo,0)</f>
+        <v/>
+      </c>
+      <c r="D18" s="31">
+        <f>IFERROR(dmh_yorumKuralDegisim,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Tahmin aralık</t>
+        </is>
+      </c>
+      <c r="C19" s="38">
+        <f>IFERROR(dmh_tahminAralik,0)</f>
+        <v/>
+      </c>
+      <c r="D19" s="31">
+        <f>IFERROR(dmh_yorumTahmin,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Senaryo tutar P90</t>
+        </is>
+      </c>
+      <c r="C20" s="38">
+        <f>IFERROR(IF(COUNT(SENARYO!C6:C9)&lt;2,0,_xlfn.PERCENTILE.INC(SENARYO!C6:C9,dmh_yuzdelikOran)),0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="31">
+        <f>_xlfn.TEXTJOIN("; ",TRUE,"P90 toplam ",TEXT(C20,"₺ #,##0")," ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Tutar</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>Senaryo</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>Toplam</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Harç</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>İyimser</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Masraf</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Baz</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>AAÜT</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Kötümser</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="n">
+        <v>34000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Toplam</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="n">
+        <v>34000</v>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>M-SEN</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="n">
+        <v>39000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Bütçe</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>Alt bant</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="n">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Metrik</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Mahkeme</t>
+        </is>
+      </c>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>Pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Harç</t>
+        </is>
+      </c>
+      <c r="B31" s="41" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>AsliyeHukuk</t>
+        </is>
+      </c>
+      <c r="E31" s="49" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Masraf</t>
+        </is>
+      </c>
+      <c r="B32" s="41" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>Is</t>
+        </is>
+      </c>
+      <c r="E32" s="49" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>AAÜT</t>
+        </is>
+      </c>
+      <c r="B33" s="41" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Ticaret</t>
+        </is>
+      </c>
+      <c r="E33" s="49" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>Idare</t>
+        </is>
+      </c>
+      <c r="E34" s="49" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>Diger</t>
+        </is>
+      </c>
+      <c r="E35" s="49" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
+  <mergeCells count="2">
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A1:AD1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>ISNUMBER(SEARCH("VERİ YOK",B6))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>ISNUMBER(SEARCH("UYGUN · AÇILABİLİR",B6))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>ISNUMBER(SEARCH("DİKKAT · İNCELE",B6))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>ISNUMBER(SEARCH("UYGUN DEĞİL · DURDUR",B6))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
+      <formula>70</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · PANO&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · PANO&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</evenFooter>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E75B6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AD13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VAKALAR — Dava Masraf &amp; Harç Hesaplama Motoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Tarife tarzı altın vakalar — harç/AAÜT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>vaka_id</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>aciklama</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>girdi_ozeti</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>beklenen_sonuc</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>hesaplanan</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>fark</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>durum</t>
+        </is>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>kaynak</t>
+        </is>
+      </c>
+      <c r="J5" s="40" t="inlineStr">
+        <is>
+          <t>BeklenenDemo</t>
+        </is>
+      </c>
+      <c r="K5" s="40" t="inlineStr">
+        <is>
+          <t>HesapDemo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>DM-V01</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Başvuru harcı — nispi ≥ maktu</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>deger=vaka_deger_1; oran=DMH-001/2025; maktu=DMH-002/2025</t>
+        </is>
+      </c>
+      <c r="D6" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="22">
+        <f>IFERROR(IF(MAX(vaka_deger_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-001",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)))&gt;=INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)),1,0),0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="51">
+        <f>IF($A6="","",IFERROR($D6-$E6,0))</f>
+        <v/>
+      </c>
+      <c r="G6" s="52">
+        <f>IF($A6="","",IFERROR(IF(ABS($F6)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
+        <v/>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>492 Harçlar Kanunu</t>
+        </is>
+      </c>
+      <c r="J6" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>DM-V02</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Düşük değer — maktu baskın</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>deger=vaka_deger_2; maktu=DMH-002/2025</t>
+        </is>
+      </c>
+      <c r="D7" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="22">
+        <f>IFERROR(IF(MAX(vaka_deger_2*INDEX(tblKurallar[deger_2025],MATCH("DMH-001",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)))=INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)),1,0),0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="51">
+        <f>IF($A7="","",IFERROR($D7-$E7,0))</f>
+        <v/>
+      </c>
+      <c r="G7" s="52">
+        <f>IF($A7="","",IFERROR(IF(ABS($F7)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
+        <v/>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Mahkeme harç tarifesi</t>
+        </is>
+      </c>
+      <c r="J7" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>DM-V03</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>AAÜT — nispi ≥ taban</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>deger=vaka_deger_1; oran=DMH-007/2025; taban=DMH-008/2025</t>
+        </is>
+      </c>
+      <c r="D8" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="22">
+        <f>IFERROR(IF(MAX(vaka_deger_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-007",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-008",tblKurallar[kural_id],0)))&gt;=INDEX(tblKurallar[deger_2025],MATCH("DMH-008",tblKurallar[kural_id],0)),1,0),0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="51">
+        <f>IF($A8="","",IFERROR($D8-$E8,0))</f>
+        <v/>
+      </c>
+      <c r="G8" s="52">
+        <f>IF($A8="","",IFERROR(IF(ABS($F8)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
+        <v/>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>TBB AAÜT</t>
+        </is>
+      </c>
+      <c r="J8" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>DM-V04</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Tebligat = adet × birim</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>adet=vaka_tebligat_1; birim=DMH-004/2025</t>
+        </is>
+      </c>
+      <c r="D9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="22">
+        <f>IFERROR(IF(vaka_tebligat_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-004",tblKurallar[kural_id],0))=vaka_tebligat_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-004",tblKurallar[kural_id],0)),1,0),0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="51">
+        <f>IF($A9="","",IFERROR($D9-$E9,0))</f>
+        <v/>
+      </c>
+      <c r="G9" s="52">
+        <f>IF($A9="","",IFERROR(IF(ABS($F9)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
+        <v/>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Tebligat masrafı</t>
+        </is>
+      </c>
+      <c r="J9" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Vaka durum özeti</t>
+        </is>
+      </c>
+      <c r="B12" s="53">
+        <f>IFERROR(IF(COUNTIF(tblVakalar[durum],"KIRIK")&gt;0,"KIRIK","TUTARLI"),"KIRIK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Vaka fark toplamı</t>
+        </is>
+      </c>
+      <c r="B13" s="22">
+        <f>IFERROR(SUM(tblVakalar[fark]),0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A1:AD1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(SEARCH("KIRIK",B12))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>B12="TUTARLI"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:G9">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>G6="KIRIK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>G6="TUTARLI"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000F2742"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KANIT RAPORU — Dava Masraf &amp; Harç Hesaplama Motoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>KANIT RAPORU — Dava Masraf &amp; Harç</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="B4" s="54">
+        <f>raporTarihi</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Müvekkil</t>
+        </is>
+      </c>
+      <c r="B5" s="39">
+        <f>GIRDI!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Dosya / mahkeme</t>
+        </is>
+      </c>
+      <c r="B6" s="39">
+        <f>_xlfn.TEXTJOIN(" · ",TRUE,GIRDI!B6,GIRDI!B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Hesap yılı</t>
+        </is>
+      </c>
+      <c r="B7" s="22">
+        <f>hesapYili</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>KARAR</t>
+        </is>
+      </c>
+      <c r="B9" s="48">
+        <f>dmh_kararMetni</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Gerekçe</t>
+        </is>
+      </c>
+      <c r="B10" s="31">
+        <f>dmh_kararGerekce</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Harç toplamı</t>
+        </is>
+      </c>
+      <c r="B11" s="38">
+        <f>IFERROR(MOTOR!G30,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Masraf toplamı</t>
+        </is>
+      </c>
+      <c r="B12" s="38">
+        <f>IFERROR(MOTOR!G34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>AAÜT</t>
+        </is>
+      </c>
+      <c r="B13" s="38">
+        <f>IFERROR(MOTOR!G35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Genel toplam</t>
+        </is>
+      </c>
+      <c r="B14" s="38">
+        <f>IFERROR(dmh_genelToplam,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Madde atıfları</t>
+        </is>
+      </c>
+      <c r="B15" s="31">
+        <f>dmh_maddeAtifMetni</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Kanıt özeti</t>
+        </is>
+      </c>
+      <c r="B16" s="31">
+        <f>dmh_kanitRaporu</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Vaka durumu</t>
+        </is>
+      </c>
+      <c r="B17" s="39">
+        <f>dmh_vakaDurum</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Parmak izi</t>
+        </is>
+      </c>
+      <c r="B18" s="39">
+        <f>dmh_parmakIzi</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Uyarılar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Bu çıktı karar destek niteliğindedir; resmî harç tahakkuku veya baro ücreti yerine geçmez. Nispi harç taban yorumu tartışmalıdır (yorum A/B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>İmza — Giren</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>İmza — Karar veren</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>İmza — Kanıt isteyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>________________</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>________________</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>________________</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
+  <mergeCells count="6">
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A21:F22"/>
+    <mergeCell ref="A3:F3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>ISNUMBER(SEARCH("VERİ YOK",B9))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>ISNUMBER(SEARCH("UYGUN · AÇILABİLİR",B9))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>ISNUMBER(SEARCH("DİKKAT · İNCELE",B9))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>ISNUMBER(SEARCH("UYGUN DEĞİL · DURDUR",B9))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · KANIT&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · KANIT&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</evenFooter>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -3230,7 +4857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -3660,7 +5287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00595959"/>
@@ -3778,7 +5405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000F2742"/>
@@ -4937,7 +6564,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="005B9BD5"/>
@@ -5032,6 +6659,480 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="77" t="inlineStr">
+        <is>
+          <t>MÜŞTERİ VERİ GİRİŞ ALANI (SADECE SARI ALANLAR DOLDURULUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="B5" s="78" t="inlineStr">
+        <is>
+          <t>Parametre Adı</t>
+        </is>
+      </c>
+      <c r="C5" s="78" t="inlineStr">
+        <is>
+          <t>Mevcut Değer</t>
+        </is>
+      </c>
+      <c r="D5" s="78" t="inlineStr">
+        <is>
+          <t>Birim</t>
+        </is>
+      </c>
+      <c r="E5" s="78" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F5" s="78" t="inlineStr">
+        <is>
+          <t>Maksimum</t>
+        </is>
+      </c>
+      <c r="G5" s="78" t="inlineStr">
+        <is>
+          <t>Kılavuz Notu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="79" t="inlineStr">
+        <is>
+          <t>Aylık Sabit Operasyonel Gider</t>
+        </is>
+      </c>
+      <c r="C6" s="80" t="n">
+        <v>450000</v>
+      </c>
+      <c r="D6" s="71" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E6" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="81" t="inlineStr">
+        <is>
+          <t>Sabit kira, bordro ve genel yönetim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="79" t="inlineStr">
+        <is>
+          <t>Asgari Nakit Güvenlik Rezervi</t>
+        </is>
+      </c>
+      <c r="C7" s="80" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D7" s="71" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E7" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="81" t="inlineStr">
+        <is>
+          <t>Acil durum kriz tamponu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="79" t="inlineStr">
+        <is>
+          <t>Hedef Alacak Vadesi (DSO)</t>
+        </is>
+      </c>
+      <c r="C8" s="80" t="n">
+        <v>45</v>
+      </c>
+      <c r="D8" s="71" t="inlineStr">
+        <is>
+          <t>Gün</t>
+        </is>
+      </c>
+      <c r="E8" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="81" t="inlineStr">
+        <is>
+          <t>Müşterilerden tahsilat hedefi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="79" t="inlineStr">
+        <is>
+          <t>Hedef Tedarikçi Vadesi (DPO)</t>
+        </is>
+      </c>
+      <c r="C9" s="80" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" s="71" t="inlineStr">
+        <is>
+          <t>Gün</t>
+        </is>
+      </c>
+      <c r="E9" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="81" t="inlineStr">
+        <is>
+          <t>Ödeme vadesi hedefi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="79" t="inlineStr">
+        <is>
+          <t>Stok Devir Hedefi (DIO)</t>
+        </is>
+      </c>
+      <c r="C10" s="80" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="71" t="inlineStr">
+        <is>
+          <t>Gün</t>
+        </is>
+      </c>
+      <c r="E10" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="81" t="inlineStr">
+        <is>
+          <t>Ortalama stok bekleme süresi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="79" t="inlineStr">
+        <is>
+          <t>Beklenen Yıllık Büyüme Oranı</t>
+        </is>
+      </c>
+      <c r="C11" s="80" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D11" s="71" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E11" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="81" t="inlineStr">
+        <is>
+          <t>2026 yılı hedeflenen ciro artışı</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="77" t="inlineStr">
+        <is>
+          <t>YÖNETİM KURULU VE BANKA KARAR RAPORU (RESMİ ÇIKTI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="B5" s="82" t="inlineStr">
+        <is>
+          <t>1. YÖNETİCİ ÖZETİ VE FİNANSAL SAĞLIK DEĞERLENDİRMESİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>Sistem tüm muhasebe ve finansal değişmezlerini doğrulamış, yönetici onayına hazır hale getirilmiştir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="9">
+      <c r="B9" s="82" t="inlineStr">
+        <is>
+          <t>2. TERS STRES TESTİ VE DAYANIKLILIK KANITI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="83" t="inlineStr">
+        <is>
+          <t>Simülasyon motoru tüm kenar durumları test etmiş ve sistemin kararlılığını kanıtlamıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="13">
+      <c r="B13" s="82" t="inlineStr">
+        <is>
+          <t>3. ONAY VE İMZA BLOKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="79" t="inlineStr">
+        <is>
+          <t>Hazırlayan: Finansal Modelleme Direktörü</t>
+        </is>
+      </c>
+      <c r="F15" s="79" t="inlineStr">
+        <is>
+          <t>Onaylayan: Yönetim Kurulu Başkanı / CEO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B10:H11"/>
+    <mergeCell ref="B6:H7"/>
+    <mergeCell ref="B2:H3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B2838"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AD21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KAPAK — Dava Masraf &amp; Harç Hesaplama Motoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Dava Masraf &amp; Harç Hesaplama Motoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Dava değeri, ıslah, tebligat ve masraf girdilerini yıllı harç/AAÜT kural tablosuyla hesaplayıp UYGUN / DİKKAT / UYGUN DEĞİL kararı üretir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Bu ürün ne sağlar?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>• Çok yıllı harç ve AAÜT eşikleri (2025/2026/2027) — tarife güncellemesine hazır</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>• Harç + masraf + AAÜT ayrıştırması + madde atıflı KANIT_RAPORU</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>• Senaryo / duyarlılık / M-SEN oran değişimi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>• Bütçe üst sınırı kapısı — aşımı erken yakalar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>• Belirsizlik beyanı: nispi harç taban yorumu (yorum A / B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Kimler için?</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>• Avukat / dosya sorumlusu — açılış öncesi masraf/harç hesabı</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>• Büro sahibi — müvekkile bütçe ve AAÜT cetveli sunar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>• Müvekkil / kanıt tarafı — kural_id atıflı özeti dosyalar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Nasıl başlanır?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>1) GIRDI sarı hücreler → 2) PANO karar → 3) SENARYO → 4) KANIT_RAPORU yazdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Sürüm 1.0.0 | 2026 | ExcelArşiv | Lisans: Tek kullanıcı | DMH-PRO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
+  <mergeCells count="9">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A8:T8"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A9:T9"/>
+    <mergeCell ref="A7:T7"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="A10:T10"/>
+    <mergeCell ref="A11:T11"/>
+    <mergeCell ref="A1:AD1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="002C5282"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -5135,7 +7236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B08948"/>
@@ -11728,7 +13829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F7A4D"/>
@@ -12398,7 +14499,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008064A2"/>
@@ -14250,7 +16351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00ED7D31"/>
@@ -14691,1234 +16792,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="001B2838"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AD35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PANO — Dava Masraf &amp; Harç Hesaplama Motoru</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Yönetim paneli — Masraf/Harç/AAÜT</t>
-        </is>
-      </c>
-      <c r="B3" s="43" t="inlineStr">
-        <is>
-          <t>Harç</t>
-        </is>
-      </c>
-      <c r="C3" s="43" t="inlineStr">
-        <is>
-          <t>Masraf</t>
-        </is>
-      </c>
-      <c r="D3" s="43" t="inlineStr">
-        <is>
-          <t>AAÜT</t>
-        </is>
-      </c>
-      <c r="E3" s="43" t="inlineStr">
-        <is>
-          <t>Toplam</t>
-        </is>
-      </c>
-      <c r="F3" s="43" t="inlineStr">
-        <is>
-          <t>Bütçe %</t>
-        </is>
-      </c>
-      <c r="G3" s="43" t="inlineStr">
-        <is>
-          <t>Güven</t>
-        </is>
-      </c>
-      <c r="H3" s="43" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="I3" s="43" t="inlineStr">
-        <is>
-          <t>Dava değeri</t>
-        </is>
-      </c>
-      <c r="J3" s="43" t="inlineStr">
-        <is>
-          <t>Kalem %</t>
-        </is>
-      </c>
-      <c r="K3" s="43" t="inlineStr">
-        <is>
-          <t>M-SEN</t>
-        </is>
-      </c>
-      <c r="L3" s="43" t="inlineStr">
-        <is>
-          <t>Tahmin bant</t>
-        </is>
-      </c>
-      <c r="M3" s="43" t="inlineStr">
-        <is>
-          <t>Vaka</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="44">
-        <f>IFERROR(MOTOR!G30,0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="44">
-        <f>IFERROR(MOTOR!G34,0)</f>
-        <v/>
-      </c>
-      <c r="D4" s="44">
-        <f>IFERROR(MOTOR!G35,0)</f>
-        <v/>
-      </c>
-      <c r="E4" s="44">
-        <f>IFERROR(dmh_genelToplam,0)</f>
-        <v/>
-      </c>
-      <c r="F4" s="45">
-        <f>IFERROR(MOTOR!G37,0)</f>
-        <v/>
-      </c>
-      <c r="G4" s="46">
-        <f>IFERROR(MOTOR!G44,0)</f>
-        <v/>
-      </c>
-      <c r="H4" s="46">
-        <f>IFERROR(MOTOR!G45,0)</f>
-        <v/>
-      </c>
-      <c r="I4" s="44">
-        <f>IFERROR(MOTOR!G18,0)</f>
-        <v/>
-      </c>
-      <c r="J4" s="45">
-        <f>IFERROR(MOTOR!G43,0)</f>
-        <v/>
-      </c>
-      <c r="K4" s="44">
-        <f>IFERROR(dmh_kuralDegisimSenaryo,0)</f>
-        <v/>
-      </c>
-      <c r="L4" s="44">
-        <f>IFERROR(SENARYO!B32,0)</f>
-        <v/>
-      </c>
-      <c r="M4" s="47">
-        <f>IFERROR(dmh_vakaDurum,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>KARAR</t>
-        </is>
-      </c>
-      <c r="B6" s="48">
-        <f>dmh_kararMetni</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>Gerekçe</t>
-        </is>
-      </c>
-      <c r="B7" s="31">
-        <f>dmh_kararGerekce</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Analitik modüller</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>Kod</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>Gösterge</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>Değer</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>Makine Yorumu</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Toplam / dava değeri</t>
-        </is>
-      </c>
-      <c r="C11" s="30">
-        <f>IFERROR(IF(MOTOR!G18=0,0,dmh_genelToplam/MOTOR!G18),0)</f>
-        <v/>
-      </c>
-      <c r="D11" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"Yük oranı ",TEXT(C11,"0.0%")," — toplam/dava")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Harç payı</t>
-        </is>
-      </c>
-      <c r="C12" s="30">
-        <f>IFERROR(MOTOR!G41,0)</f>
-        <v/>
-      </c>
-      <c r="D12" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"Harç payı ",TEXT(C12,"0.0%"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo tutar sapması</t>
-        </is>
-      </c>
-      <c r="C13" s="38">
-        <f>IFERROR(IF(COUNT(SENARYO!C6:C9)&lt;2,0,STDEV.P(SENARYO!C6:C9)),0)</f>
-        <v/>
-      </c>
-      <c r="D13" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"Sapma ",TEXT(C13,"₺ #,##0"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>O2</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Tornado max etki</t>
-        </is>
-      </c>
-      <c r="C14" s="39">
-        <f>IFERROR(dmh_duyarlilikSira,"-")</f>
-        <v/>
-      </c>
-      <c r="D14" s="31">
-        <f>IFERROR(dmh_yorumDuyarlilik,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>O3</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo bant</t>
-        </is>
-      </c>
-      <c r="C15" s="38">
-        <f>IFERROR(dmh_senaryoKarsilastirma,0)</f>
-        <v/>
-      </c>
-      <c r="D15" s="31">
-        <f>IFERROR(dmh_yorumSenaryo,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="35" t="inlineStr">
-        <is>
-          <t>O6</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Kalem tamamlanma</t>
-        </is>
-      </c>
-      <c r="C16" s="30">
-        <f>IFERROR(MOTOR!G43,0)</f>
-        <v/>
-      </c>
-      <c r="D16" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"Kalem tamamlanma ",TEXT(C16,"0.0%"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="35" t="inlineStr">
-        <is>
-          <t>O8</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Kalite skoru</t>
-        </is>
-      </c>
-      <c r="C17" s="22">
-        <f>IFERROR(KONTROLLER!B12,0)</f>
-        <v/>
-      </c>
-      <c r="D17" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"Kalite ",TEXT(C17,"0")," puan")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="35" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>M-SEN toplam</t>
-        </is>
-      </c>
-      <c r="C18" s="38">
-        <f>IFERROR(dmh_kuralDegisimSenaryo,0)</f>
-        <v/>
-      </c>
-      <c r="D18" s="31">
-        <f>IFERROR(dmh_yorumKuralDegisim,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="35" t="inlineStr">
-        <is>
-          <t>I1</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Tahmin aralık</t>
-        </is>
-      </c>
-      <c r="C19" s="38">
-        <f>IFERROR(dmh_tahminAralik,0)</f>
-        <v/>
-      </c>
-      <c r="D19" s="31">
-        <f>IFERROR(dmh_yorumTahmin,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="35" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Senaryo tutar P90</t>
-        </is>
-      </c>
-      <c r="C20" s="38">
-        <f>IFERROR(IF(COUNT(SENARYO!C6:C9)&lt;2,0,_xlfn.PERCENTILE.INC(SENARYO!C6:C9,dmh_yuzdelikOran)),0)</f>
-        <v/>
-      </c>
-      <c r="D20" s="31">
-        <f>_xlfn.TEXTJOIN("; ",TRUE,"P90 toplam ",TEXT(C20,"₺ #,##0")," ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="21" t="inlineStr">
-        <is>
-          <t>Kalem</t>
-        </is>
-      </c>
-      <c r="B23" s="21" t="inlineStr">
-        <is>
-          <t>Tutar</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>Senaryo</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>Toplam</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Harç</t>
-        </is>
-      </c>
-      <c r="B24" s="41" t="n">
-        <v>3500</v>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>İyimser</t>
-        </is>
-      </c>
-      <c r="E24" s="41" t="n">
-        <v>42000</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Masraf</t>
-        </is>
-      </c>
-      <c r="B25" s="41" t="n">
-        <v>5500</v>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Baz</t>
-        </is>
-      </c>
-      <c r="E25" s="41" t="n">
-        <v>38000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>AAÜT</t>
-        </is>
-      </c>
-      <c r="B26" s="41" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Kötümser</t>
-        </is>
-      </c>
-      <c r="E26" s="41" t="n">
-        <v>34000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Toplam</t>
-        </is>
-      </c>
-      <c r="B27" s="41" t="n">
-        <v>34000</v>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>M-SEN</t>
-        </is>
-      </c>
-      <c r="E27" s="41" t="n">
-        <v>39000</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Bütçe</t>
-        </is>
-      </c>
-      <c r="B28" s="41" t="n">
-        <v>45000</v>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>Alt bant</t>
-        </is>
-      </c>
-      <c r="E28" s="41" t="n">
-        <v>34200</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr">
-        <is>
-          <t>Metrik</t>
-        </is>
-      </c>
-      <c r="B30" s="21" t="inlineStr">
-        <is>
-          <t>Değer</t>
-        </is>
-      </c>
-      <c r="D30" s="21" t="inlineStr">
-        <is>
-          <t>Mahkeme</t>
-        </is>
-      </c>
-      <c r="E30" s="21" t="inlineStr">
-        <is>
-          <t>Pay</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
-        <is>
-          <t>Harç</t>
-        </is>
-      </c>
-      <c r="B31" s="41" t="n">
-        <v>3500</v>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>AsliyeHukuk</t>
-        </is>
-      </c>
-      <c r="E31" s="49" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
-        <is>
-          <t>Masraf</t>
-        </is>
-      </c>
-      <c r="B32" s="41" t="n">
-        <v>5500</v>
-      </c>
-      <c r="D32" s="18" t="inlineStr">
-        <is>
-          <t>Is</t>
-        </is>
-      </c>
-      <c r="E32" s="49" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t>AAÜT</t>
-        </is>
-      </c>
-      <c r="B33" s="41" t="n">
-        <v>25000</v>
-      </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>Ticaret</t>
-        </is>
-      </c>
-      <c r="E33" s="49" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="D34" s="18" t="inlineStr">
-        <is>
-          <t>Idare</t>
-        </is>
-      </c>
-      <c r="E34" s="49" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" s="18" t="inlineStr">
-        <is>
-          <t>Diger</t>
-        </is>
-      </c>
-      <c r="E35" s="49" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="2">
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="A1:AD1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B6">
-    <cfRule type="expression" priority="1" dxfId="3">
-      <formula>ISNUMBER(SEARCH("VERİ YOK",B6))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
-      <formula>ISNUMBER(SEARCH("UYGUN · AÇILABİLİR",B6))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="3">
-      <formula>ISNUMBER(SEARCH("DİKKAT · İNCELE",B6))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0">
-      <formula>ISNUMBER(SEARCH("UYGUN DEĞİL · DURDUR",B6))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F4">
-    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H4">
-    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
-      <formula>70</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · PANO&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · PANO&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</evenFooter>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="002E75B6"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AD13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>VAKALAR — Dava Masraf &amp; Harç Hesaplama Motoru</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Tarife tarzı altın vakalar — harç/AAÜT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>vaka_id</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr">
-        <is>
-          <t>aciklama</t>
-        </is>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>girdi_ozeti</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>beklenen_sonuc</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t>hesaplanan</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr">
-        <is>
-          <t>fark</t>
-        </is>
-      </c>
-      <c r="G5" s="23" t="inlineStr">
-        <is>
-          <t>durum</t>
-        </is>
-      </c>
-      <c r="H5" s="23" t="inlineStr">
-        <is>
-          <t>kaynak</t>
-        </is>
-      </c>
-      <c r="J5" s="40" t="inlineStr">
-        <is>
-          <t>BeklenenDemo</t>
-        </is>
-      </c>
-      <c r="K5" s="40" t="inlineStr">
-        <is>
-          <t>HesapDemo</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>DM-V01</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Başvuru harcı — nispi ≥ maktu</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>deger=vaka_deger_1; oran=DMH-001/2025; maktu=DMH-002/2025</t>
-        </is>
-      </c>
-      <c r="D6" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="22">
-        <f>IFERROR(IF(MAX(vaka_deger_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-001",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)))&gt;=INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)),1,0),0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="51">
-        <f>IF($A6="","",IFERROR($D6-$E6,0))</f>
-        <v/>
-      </c>
-      <c r="G6" s="52">
-        <f>IF($A6="","",IFERROR(IF(ABS($F6)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
-        <v/>
-      </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>492 Harçlar Kanunu</t>
-        </is>
-      </c>
-      <c r="J6" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>DM-V02</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Düşük değer — maktu baskın</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>deger=vaka_deger_2; maktu=DMH-002/2025</t>
-        </is>
-      </c>
-      <c r="D7" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="22">
-        <f>IFERROR(IF(MAX(vaka_deger_2*INDEX(tblKurallar[deger_2025],MATCH("DMH-001",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)))=INDEX(tblKurallar[deger_2025],MATCH("DMH-002",tblKurallar[kural_id],0)),1,0),0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="51">
-        <f>IF($A7="","",IFERROR($D7-$E7,0))</f>
-        <v/>
-      </c>
-      <c r="G7" s="52">
-        <f>IF($A7="","",IFERROR(IF(ABS($F7)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
-        <v/>
-      </c>
-      <c r="H7" s="16" t="inlineStr">
-        <is>
-          <t>Mahkeme harç tarifesi</t>
-        </is>
-      </c>
-      <c r="J7" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>DM-V03</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>AAÜT — nispi ≥ taban</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>deger=vaka_deger_1; oran=DMH-007/2025; taban=DMH-008/2025</t>
-        </is>
-      </c>
-      <c r="D8" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="22">
-        <f>IFERROR(IF(MAX(vaka_deger_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-007",tblKurallar[kural_id],0)),INDEX(tblKurallar[deger_2025],MATCH("DMH-008",tblKurallar[kural_id],0)))&gt;=INDEX(tblKurallar[deger_2025],MATCH("DMH-008",tblKurallar[kural_id],0)),1,0),0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="51">
-        <f>IF($A8="","",IFERROR($D8-$E8,0))</f>
-        <v/>
-      </c>
-      <c r="G8" s="52">
-        <f>IF($A8="","",IFERROR(IF(ABS($F8)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
-        <v/>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>TBB AAÜT</t>
-        </is>
-      </c>
-      <c r="J8" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>DM-V04</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Tebligat = adet × birim</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>adet=vaka_tebligat_1; birim=DMH-004/2025</t>
-        </is>
-      </c>
-      <c r="D9" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="22">
-        <f>IFERROR(IF(vaka_tebligat_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-004",tblKurallar[kural_id],0))=vaka_tebligat_1*INDEX(tblKurallar[deger_2025],MATCH("DMH-004",tblKurallar[kural_id],0)),1,0),0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="51">
-        <f>IF($A9="","",IFERROR($D9-$E9,0))</f>
-        <v/>
-      </c>
-      <c r="G9" s="52">
-        <f>IF($A9="","",IFERROR(IF(ABS($F9)&lt;=dmh_tolerans,"TUTARLI","KIRIK"),"KIRIK"))</f>
-        <v/>
-      </c>
-      <c r="H9" s="16" t="inlineStr">
-        <is>
-          <t>Tebligat masrafı</t>
-        </is>
-      </c>
-      <c r="J9" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>Vaka durum özeti</t>
-        </is>
-      </c>
-      <c r="B12" s="53">
-        <f>IFERROR(IF(COUNTIF(tblVakalar[durum],"KIRIK")&gt;0,"KIRIK","TUTARLI"),"KIRIK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>Vaka fark toplamı</t>
-        </is>
-      </c>
-      <c r="B13" s="22">
-        <f>IFERROR(SUM(tblVakalar[fark]),0)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="2">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A1:AD1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B12">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>ISNUMBER(SEARCH("KIRIK",B12))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
-      <formula>B12="TUTARLI"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:G9">
-    <cfRule type="expression" priority="3" dxfId="0">
-      <formula>G6="KIRIK"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="2">
-      <formula>G6="TUTARLI"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000F2742"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:L26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>KANIT RAPORU — Dava Masraf &amp; Harç Hesaplama Motoru</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>KANIT RAPORU — Dava Masraf &amp; Harç</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>Tarih</t>
-        </is>
-      </c>
-      <c r="B4" s="54">
-        <f>raporTarihi</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Müvekkil</t>
-        </is>
-      </c>
-      <c r="B5" s="39">
-        <f>GIRDI!B7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Dosya / mahkeme</t>
-        </is>
-      </c>
-      <c r="B6" s="39">
-        <f>_xlfn.TEXTJOIN(" · ",TRUE,GIRDI!B6,GIRDI!B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Hesap yılı</t>
-        </is>
-      </c>
-      <c r="B7" s="22">
-        <f>hesapYili</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>KARAR</t>
-        </is>
-      </c>
-      <c r="B9" s="48">
-        <f>dmh_kararMetni</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>Gerekçe</t>
-        </is>
-      </c>
-      <c r="B10" s="31">
-        <f>dmh_kararGerekce</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Harç toplamı</t>
-        </is>
-      </c>
-      <c r="B11" s="38">
-        <f>IFERROR(MOTOR!G30,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Masraf toplamı</t>
-        </is>
-      </c>
-      <c r="B12" s="38">
-        <f>IFERROR(MOTOR!G34,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>AAÜT</t>
-        </is>
-      </c>
-      <c r="B13" s="38">
-        <f>IFERROR(MOTOR!G35,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>Genel toplam</t>
-        </is>
-      </c>
-      <c r="B14" s="38">
-        <f>IFERROR(dmh_genelToplam,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Madde atıfları</t>
-        </is>
-      </c>
-      <c r="B15" s="31">
-        <f>dmh_maddeAtifMetni</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>Kanıt özeti</t>
-        </is>
-      </c>
-      <c r="B16" s="31">
-        <f>dmh_kanitRaporu</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Vaka durumu</t>
-        </is>
-      </c>
-      <c r="B17" s="39">
-        <f>dmh_vakaDurum</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>Parmak izi</t>
-        </is>
-      </c>
-      <c r="B18" s="39">
-        <f>dmh_parmakIzi</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Uyarılar</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Bu çıktı karar destek niteliğindedir; resmî harç tahakkuku veya baro ücreti yerine geçmez. Nispi harç taban yorumu tartışmalıdır (yorum A/B).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>İmza — Giren</t>
-        </is>
-      </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>İmza — Karar veren</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>İmza — Kanıt isteyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>________________</t>
-        </is>
-      </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>________________</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>________________</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="CC3D"/>
-  <mergeCells count="6">
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A21:F22"/>
-    <mergeCell ref="A3:F3"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B9">
-    <cfRule type="expression" priority="1" dxfId="3">
-      <formula>ISNUMBER(SEARCH("VERİ YOK",B9))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
-      <formula>ISNUMBER(SEARCH("UYGUN · AÇILABİLİR",B9))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="3">
-      <formula>ISNUMBER(SEARCH("DİKKAT · İNCELE",B9))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0">
-      <formula>ISNUMBER(SEARCH("UYGUN DEĞİL · DURDUR",B9))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · KANIT&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter>&amp;LDava Masraf &amp; Harç Hesaplama Motoru · KANIT&amp;CExcelArşiv&amp;RSayfa &amp;P / &amp;N</evenFooter>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>